<commit_message>
update script to fetch, display data, and write data to Excel file for both sub-accounts
</commit_message>
<xml_diff>
--- a/ExcelFiles/account_info.xlsx
+++ b/ExcelFiles/account_info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danagershon/Documents/Investing/ExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E03B91B3-7CE7-7249-BC39-8E7BBA53BF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF29B839-2477-8E44-8FBA-F4E5A211EBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="25460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="25440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
   <si>
     <t>Date</t>
   </si>
@@ -28,6 +28,9 @@
     <t>Exchange Rate</t>
   </si>
   <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Net Liquidation</t>
   </si>
   <si>
@@ -58,17 +61,25 @@
     <t>%</t>
   </si>
   <si>
-    <t>2024-06-27 21:54:50</t>
+    <t>2024-10-06 19:46:26</t>
+  </si>
+  <si>
+    <t>Sum of Accounts</t>
+  </si>
+  <si>
+    <t>U13834548</t>
+  </si>
+  <si>
+    <t>U19254019</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="\₪#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="%#,##0.00"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="\$#,##0"/>
+    <numFmt numFmtId="165" formatCode="\₪#,##0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -132,9 +143,7 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -145,7 +154,9 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -159,13 +170,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -480,93 +491,82 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.15">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="6" t="s">
+      <c r="E1" s="8"/>
+      <c r="F1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="7"/>
-      <c r="I1" s="6" t="s">
+      <c r="G1" s="8"/>
+      <c r="H1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="7"/>
-      <c r="K1" s="6" t="s">
+      <c r="I1" s="8"/>
+      <c r="J1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="M1" s="7"/>
-      <c r="N1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="O1" s="6" t="s">
+      <c r="N1" s="8"/>
+      <c r="O1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="8"/>
+      <c r="P1" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="Q1" s="7"/>
+      <c r="R1" s="8"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.15">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
-      <c r="C2" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C2" s="5"/>
       <c r="D2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>10</v>
@@ -574,78 +574,168 @@
       <c r="M2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="N2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="5"/>
       <c r="P2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>11</v>
       </c>
+      <c r="R2" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3">
-        <v>3.7570000000000001</v>
-      </c>
-      <c r="C3" s="1">
-        <v>23520</v>
-      </c>
-      <c r="D3" s="2">
-        <v>88365</v>
-      </c>
-      <c r="E3" s="1">
-        <v>21084</v>
-      </c>
-      <c r="F3" s="2">
-        <v>79213</v>
-      </c>
-      <c r="G3" s="1">
-        <v>2399</v>
-      </c>
-      <c r="H3" s="2">
-        <v>9013</v>
-      </c>
-      <c r="I3" s="1">
-        <v>36</v>
-      </c>
-      <c r="J3" s="2">
-        <v>135</v>
-      </c>
-      <c r="K3" s="1">
-        <v>-266</v>
-      </c>
-      <c r="L3" s="2">
-        <v>-999</v>
-      </c>
-      <c r="M3" s="3">
-        <v>-1.118304885226604E-2</v>
-      </c>
-      <c r="N3" s="2">
+        <v>3.8140000000000001</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="1">
+        <v>24100.74</v>
+      </c>
+      <c r="E3" s="2">
+        <v>91920.22</v>
+      </c>
+      <c r="F3" s="1">
+        <v>19202.38</v>
+      </c>
+      <c r="G3" s="2">
+        <v>73237.88</v>
+      </c>
+      <c r="H3" s="1">
+        <v>4897.32</v>
+      </c>
+      <c r="I3" s="2">
+        <v>18678.38</v>
+      </c>
+      <c r="J3" s="1">
+        <v>1.04</v>
+      </c>
+      <c r="K3" s="2">
+        <v>3.97</v>
+      </c>
+      <c r="L3" s="1">
+        <v>-110.16</v>
+      </c>
+      <c r="M3" s="2">
+        <v>-420.14999999999992</v>
+      </c>
+      <c r="N3" s="3">
+        <v>-4.5500167280026768E-3</v>
+      </c>
+      <c r="O3" s="2">
         <v>86500</v>
       </c>
-      <c r="O3" s="1">
-        <v>496.40670747937179</v>
-      </c>
-      <c r="P3" s="2">
-        <v>1865</v>
-      </c>
-      <c r="Q3" s="3">
-        <v>2.15606936416185E-2</v>
-      </c>
+      <c r="P3" s="1">
+        <v>1421.1379129522811</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>5420.2200000000012</v>
+      </c>
+      <c r="R3" s="3">
+        <v>6.2661502890173429E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1">
+        <v>20958.13</v>
+      </c>
+      <c r="E4" s="2">
+        <v>79934.31</v>
+      </c>
+      <c r="F4" s="1">
+        <v>18283.16</v>
+      </c>
+      <c r="G4" s="2">
+        <v>69731.97</v>
+      </c>
+      <c r="H4" s="1">
+        <v>2674.97</v>
+      </c>
+      <c r="I4" s="2">
+        <v>10202.34</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
+        <v>340.7</v>
+      </c>
+      <c r="M4" s="2">
+        <v>1299.43</v>
+      </c>
+      <c r="N4" s="3">
+        <v>1.652485300059222E-2</v>
+      </c>
+      <c r="O4" s="2"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="3"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="1">
+        <v>3142.61</v>
+      </c>
+      <c r="E5" s="2">
+        <v>11985.91</v>
+      </c>
+      <c r="F5" s="1">
+        <v>919.22</v>
+      </c>
+      <c r="G5" s="2">
+        <v>3505.91</v>
+      </c>
+      <c r="H5" s="1">
+        <v>2222.35</v>
+      </c>
+      <c r="I5" s="2">
+        <v>8476.0400000000009</v>
+      </c>
+      <c r="J5" s="1">
+        <v>1.04</v>
+      </c>
+      <c r="K5" s="2">
+        <v>3.97</v>
+      </c>
+      <c r="L5" s="1">
+        <v>-450.86</v>
+      </c>
+      <c r="M5" s="2">
+        <v>-1719.58</v>
+      </c>
+      <c r="N5" s="3">
+        <v>-0.1254664711267939</v>
+      </c>
+      <c r="O5" s="2"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="K1:M1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="L1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>